<commit_message>
Add competitor chicken brand keywords tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0189RpT3ueNgqmUTMfiRJ2Yn
</commit_message>
<xml_diff>
--- a/curryit-amazon-keywords/CURRYiT_Chettinad_Keyword_Segregation.xlsx
+++ b/curryit-amazon-keywords/CURRYiT_Chettinad_Keyword_Segregation.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not Relevant" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Structure" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chicken Brand Keywords" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Keywords'!$A$1:$F$208</definedName>
@@ -105,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +120,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -541,7 +543,6 @@
       <c r="C5" t="n">
         <v>1980</v>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -555,7 +556,6 @@
       <c r="C6" t="n">
         <v>1490</v>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -569,7 +569,6 @@
       <c r="C7" t="n">
         <v>720</v>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -583,7 +582,6 @@
       <c r="C8" t="n">
         <v>520</v>
       </c>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -597,7 +595,6 @@
       <c r="C9" t="n">
         <v>230</v>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -611,7 +608,6 @@
       <c r="C10" t="n">
         <v>70</v>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -625,7 +621,6 @@
       <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -639,7 +634,6 @@
       <c r="C12" t="n">
         <v>18390</v>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -653,7 +647,6 @@
       <c r="C13" t="n">
         <v>190</v>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -667,7 +660,6 @@
       <c r="C14" t="n">
         <v>140</v>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -681,7 +673,6 @@
       <c r="C15" t="n">
         <v>120</v>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -695,7 +686,6 @@
       <c r="C16" t="n">
         <v>90</v>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -709,7 +699,6 @@
       <c r="C17" t="n">
         <v>70</v>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -723,7 +712,6 @@
       <c r="C18" t="n">
         <v>40</v>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -737,7 +725,6 @@
       <c r="C19" t="n">
         <v>20</v>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -751,7 +738,6 @@
       <c r="C20" t="n">
         <v>0</v>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -765,7 +751,6 @@
       <c r="C21" t="n">
         <v>0</v>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -10993,4 +10978,1476 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Avg. monthly searches</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Relevant</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Ad group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MDH</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>mdh chicken masala</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1600</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MDH</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>chicken curry masala mdh</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>140</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MDH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>mdh chicken curry masala</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>140</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MDH</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>mdh masala chicken</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MDH</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>mdh ka chicken masala</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MDH</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>mdh chicken</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MDH</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>mdh chicken curry</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr"/>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>MDH Total</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>1990</v>
+      </c>
+      <c r="D9" s="11" t="inlineStr"/>
+      <c r="E9" s="11" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Suhana</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>suhana chicken gravy masala</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Suhana</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>suhana chicken curry masala</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>90</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr"/>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Suhana Total</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>1390</v>
+      </c>
+      <c r="D12" s="11" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sunrise</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>sunrise chicken masala</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>320</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sunrise</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>sunrise chicken curry masala</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>140</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr"/>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Sunrise Total</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>460</v>
+      </c>
+      <c r="D15" s="11" t="inlineStr"/>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Aachi</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>aachi chicken</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>40</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Aachi</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>aachi chicken curry masala</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>30</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Aachi</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>aachi chettinad chicken masala</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Chettinad Competitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Aachi</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>aachi chicken varuval</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Aachi</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>aachi masala chicken gravy</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Aachi</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>chicken curry with aachi masala</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr"/>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Aachi Total</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="D22" s="11" t="inlineStr"/>
+      <c r="E22" s="11" t="inlineStr"/>
+      <c r="F22" s="11" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sakthi</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>sakthi chettinad chicken masala</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>70</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Chettinad Competitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sakthi</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>sakthi chettinad chicken masala powder</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Chettinad Competitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr"/>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Sakthi Total</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="D25" s="11" t="inlineStr"/>
+      <c r="E25" s="11" t="inlineStr"/>
+      <c r="F25" s="11" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Everest</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>everest chicken curry masala</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>50</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Everest</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>chicken curry with everest masala</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>10</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr"/>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Everest Total</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="D28" s="11" t="inlineStr"/>
+      <c r="E28" s="11" t="inlineStr"/>
+      <c r="F28" s="11" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Zoff</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>zoff chicken curry masala</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>50</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr"/>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Zoff Total</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D30" s="11" t="inlineStr"/>
+      <c r="E30" s="11" t="inlineStr"/>
+      <c r="F30" s="11" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Banne Nawab</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>banne nawab chicken masala</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>40</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Banne Nawab</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>banne nawab chicken curry</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr"/>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Banne Nawab Total</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D33" s="11" t="inlineStr"/>
+      <c r="E33" s="11" t="inlineStr"/>
+      <c r="F33" s="11" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>India Gate</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>india gate chettinad chicken masala</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>20</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Chettinad Competitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>India Gate</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>india gate classic chettinad chicken masala</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>20</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Chettinad Competitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>India Gate</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>india gate classic chettinad chicken masala gravy</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Chettinad Competitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr"/>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>India Gate Total</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D37" s="11" t="inlineStr"/>
+      <c r="E37" s="11" t="inlineStr"/>
+      <c r="F37" s="11" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Mother's Recipe</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>mother's chicken masala</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>30</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Mother's Recipe</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>mother's recipe chicken curry masala</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Mother's Recipe</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>mothers recipe chicken chettinad masala</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Chettinad Competitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr"/>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Mother's Recipe Total</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D41" s="11" t="inlineStr"/>
+      <c r="E41" s="11" t="inlineStr"/>
+      <c r="F41" s="11" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Priya</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>priya chicken masala paste</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>30</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Cooking Paste Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr"/>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>Priya Total</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D43" s="11" t="inlineStr"/>
+      <c r="E43" s="11" t="inlineStr"/>
+      <c r="F43" s="11" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Shan</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>shan chicken curry</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>10</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Shan</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>shan chicken curry masala</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr"/>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Shan Total</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D46" s="11" t="inlineStr"/>
+      <c r="E46" s="11" t="inlineStr"/>
+      <c r="F46" s="11" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Kitchens of India</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>kitchens of india chicken curry paste</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Cooking Paste Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr"/>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Kitchens of India Total</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" s="11" t="inlineStr"/>
+      <c r="E48" s="11" t="inlineStr"/>
+      <c r="F48" s="11" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Roopak</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>roopak chicken curry masala</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>10</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr"/>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Roopak Total</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D50" s="11" t="inlineStr"/>
+      <c r="E50" s="11" t="inlineStr"/>
+      <c r="F50" s="11" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Patak</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>patak chicken curry</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>10</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr"/>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Patak Total</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D52" s="11" t="inlineStr"/>
+      <c r="E52" s="11" t="inlineStr"/>
+      <c r="F52" s="11" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Eastern</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>chicken curry with eastern chicken masala</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>10</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr"/>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>Eastern Total</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D54" s="11" t="inlineStr"/>
+      <c r="E54" s="11" t="inlineStr"/>
+      <c r="F54" s="11" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Tata Sampann</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>tata sampann chicken curry masala</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr"/>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>Tata Sampann Total</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="11" t="inlineStr"/>
+      <c r="E56" s="11" t="inlineStr"/>
+      <c r="F56" s="11" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SRR</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>srr chicken curry masala</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Competitor</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Chicken Curry Masala Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr"/>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>SRR Total</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="11" t="inlineStr"/>
+      <c r="E58" s="11" t="inlineStr"/>
+      <c r="F58" s="11" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr"/>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>4340</v>
+      </c>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>